<commit_message>
Label invented inputs and record the measured eval bill.
Widen the vendored secret scanner, mark every case input as illustrative, and keep the 2026-10-17 23-case eval bills in a separate file with an estimated per-item split that is not applied.

Co-authored-by: dlescanogithub <dlescanogithub@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/results/refund-desk/model.xlsx
+++ b/docs/results/refund-desk/model.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>rationale</t>
         </is>
       </c>
@@ -476,6 +481,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>[EST] Planning volume for a mid-size fictional returns desk, not a count from a warehouse.</t>
         </is>
       </c>
@@ -496,6 +506,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>[EST] A conventional business month. It is not this company's calendar.</t>
         </is>
       </c>
@@ -516,6 +531,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>[EST] Time to read a return, check policy and type a decision without an agent.</t>
         </is>
       </c>
@@ -536,6 +556,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>[EST] Loaded desk cost, not a wage from a payroll system.</t>
         </is>
       </c>
@@ -556,6 +581,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>[EST] Share of manual decisions that need rework or a goodwill payment.</t>
         </is>
       </c>
@@ -576,6 +606,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>[EST] Residual errors after the review policy. Not a measured model score.</t>
         </is>
       </c>
@@ -596,6 +631,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>[EST] Average cost of one bad refund decision, goodwill plus rework.</t>
         </is>
       </c>
@@ -616,6 +656,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>[EST] Prompt size for one case file. Not a trace from a provider.</t>
         </is>
       </c>
@@ -636,6 +681,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>[EST] Draft length. Not a measured completion.</t>
         </is>
       </c>
@@ -656,6 +706,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>[EST] Illustrative blended price. Not copied from a vendor price page.</t>
         </is>
       </c>
@@ -676,6 +731,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>[EST] Illustrative blended price. Not copied from a vendor price page.</t>
         </is>
       </c>
@@ -696,6 +756,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>[EST] Time a person spends when a case is routed to review.</t>
         </is>
       </c>
@@ -716,6 +781,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>[EST] Share of cases a person still opens. The rest are not auto-approved by this model.</t>
         </is>
       </c>
@@ -736,6 +806,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>[EST] One-time build, integration and change-management sketch. Not a quote.</t>
         </is>
       </c>
@@ -756,6 +831,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>[EST] Fixed monthly platform and on-call cost. Charged in full during the ramp.</t>
         </is>
       </c>
@@ -776,6 +856,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>[EST] Months until the desk uses the agent on every case.</t>
         </is>
       </c>
@@ -796,6 +881,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>[EST] Annual discount rate for a 3-year NPV. Not a treasury rate.</t>
         </is>
       </c>
@@ -811,7 +901,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1 when the case is stated per month</t>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1 when the case is stated per month [EST]</t>
         </is>
       </c>
     </row>
@@ -826,7 +921,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>illustrative</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>unused in this volume mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Illustrative numbers, replace with your own</t>
         </is>
       </c>
     </row>

</xml_diff>